<commit_message>
Fix debt aging workbook failing to open in Excel
- Table columns were written as Column1..N instead of the header text, so
  Excel rejected the tables and every structured reference to them
- Data validation formulas were stored with a leading '='
- Conditional formatting used structured references, which Excel forbids
- Overlapping merged ranges on the free dashboard
- Add check_workbook.py to catch these before publishing

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HCmRdqT7qwyBh54idEMC6a
</commit_message>
<xml_diff>
--- a/Debt_Aging_Template_Free.xlsx
+++ b/Debt_Aging_Template_Free.xlsx
@@ -408,7 +408,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -507,40 +507,11 @@
         <color rgb="002C5282"/>
       </top>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00C9D3DD"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color rgb="00C9D3DD"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00C9D3DD"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="00C9D3DD"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" readingOrder="2"/>
@@ -864,10 +835,7 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1" readingOrder="2"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="28" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" indent="1" readingOrder="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="28" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" indent="1" readingOrder="2"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1209,39 +1177,39 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="tblCustomers" displayName="tblCustomers" ref="A4:Q19" headerRowCount="1">
   <autoFilter ref="A4:Q19"/>
   <tableColumns count="17">
-    <tableColumn id="1" name="Column1"/>
-    <tableColumn id="2" name="Column2"/>
-    <tableColumn id="3" name="Column3"/>
-    <tableColumn id="4" name="Column4"/>
-    <tableColumn id="5" name="Column5"/>
-    <tableColumn id="6" name="Column6"/>
-    <tableColumn id="7" name="Column7"/>
-    <tableColumn id="8" name="Column8"/>
-    <tableColumn id="9" name="Column9">
+    <tableColumn id="1" name="كود العميل"/>
+    <tableColumn id="2" name="اسم العميل"/>
+    <tableColumn id="3" name="الرقم الضريبي"/>
+    <tableColumn id="4" name="المدينة"/>
+    <tableColumn id="5" name="المندوب"/>
+    <tableColumn id="6" name="حد الائتمان"/>
+    <tableColumn id="7" name="مدة السداد"/>
+    <tableColumn id="8" name="الجوال"/>
+    <tableColumn id="9" name="الرصيد">
       <calculatedColumnFormula>ROUND(SUMIFS(tblInv[المتبقي],tblInv[كود العميل],tblCustomers[[#This Row],[كود العميل]]),2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" name="Column10">
+    <tableColumn id="10" name="المتأخر">
       <calculatedColumnFormula>ROUND(SUMIFS(tblInv[المتبقي],tblInv[كود العميل],tblCustomers[[#This Row],[كود العميل]],tblInv[أيام التأخير],"&gt;0"),2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" name="Column11">
+    <tableColumn id="11" name="استخدام الحد %">
       <calculatedColumnFormula>IFERROR(tblCustomers[[#This Row],[الرصيد]]/tblCustomers[[#This Row],[حد الائتمان]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" name="Column12">
+    <tableColumn id="12" name="أقدم فاتورة (يوم)">
       <calculatedColumnFormula>SUMPRODUCT(MAX((tblInv[كود العميل]=tblCustomers[[#This Row],[كود العميل]])*tblInv[أيام التأخير]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" name="Column13">
+    <tableColumn id="13" name="غير مخصص">
       <calculatedColumnFormula>ROUND(SUMIFS(tblRec[المبلغ],tblRec[كود العميل],tblCustomers[[#This Row],[كود العميل]],tblRec[رقم الفاتورة],"",tblRec[التاريخ],"&lt;="&amp;AsOf),2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" name="Column14">
+    <tableColumn id="14" name="الصافي">
       <calculatedColumnFormula>ROUND(tblCustomers[[#This Row],[الرصيد]]-tblCustomers[[#This Row],[غير مخصص]],2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" name="Column15">
+    <tableColumn id="15" name="مدرج">
       <calculatedColumnFormula>IF(AND(OR(tblCustomers[[#This Row],[الرصيد]]&lt;&gt;0,tblCustomers[[#This Row],[غير مخصص]]&lt;&gt;0),OR(RepF="الكل",tblCustomers[[#This Row],[المندوب]]=RepF),OR(CityF="الكل",tblCustomers[[#This Row],[المدينة]]=CityF)),1,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" name="Column16">
+    <tableColumn id="16" name="ترتيب">
       <calculatedColumnFormula>IF(tblCustomers[[#This Row],[مدرج]]=1,COUNTIFS(tblCustomers[مدرج],1,tblCustomers[الصافي],"&gt;"&amp;tblCustomers[[#This Row],[الصافي]])+COUNTIFS(INDEX(tblCustomers[مدرج],1):tblCustomers[[#This Row],[مدرج]],1,INDEX(tblCustomers[الصافي],1):tblCustomers[[#This Row],[الصافي]],tblCustomers[[#This Row],[الصافي]]),"")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" name="Column17">
+    <tableColumn id="17" name="ترتيب المتأخر">
       <calculatedColumnFormula>IF(tblCustomers[[#This Row],[المتأخر]]&gt;0,COUNTIFS(tblCustomers[المتأخر],"&gt;"&amp;tblCustomers[[#This Row],[المتأخر]])+COUNTIFS(INDEX(tblCustomers[المتأخر],1):tblCustomers[[#This Row],[المتأخر]],tblCustomers[[#This Row],[المتأخر]]),"")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1253,44 +1221,44 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="tblInv" displayName="tblInv" ref="A4:P124" headerRowCount="1">
   <autoFilter ref="A4:P124"/>
   <tableColumns count="16">
-    <tableColumn id="1" name="Column1"/>
-    <tableColumn id="2" name="Column2"/>
-    <tableColumn id="3" name="Column3"/>
-    <tableColumn id="4" name="Column4">
+    <tableColumn id="1" name="رقم الفاتورة"/>
+    <tableColumn id="2" name="تاريخ الفاتورة"/>
+    <tableColumn id="3" name="كود العميل"/>
+    <tableColumn id="4" name="اسم العميل">
       <calculatedColumnFormula>IF(tblInv[[#This Row],[كود العميل]]="","",IFERROR(INDEX(tblCustomers[اسم العميل],MATCH(tblInv[[#This Row],[كود العميل]],tblCustomers[كود العميل],0)),"⚠ كود غير موجود"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" name="Column5"/>
-    <tableColumn id="6" name="Column6">
+    <tableColumn id="5" name="المبلغ قبل الضريبة"/>
+    <tableColumn id="6" name="الضريبة">
       <calculatedColumnFormula>ROUND(tblInv[[#This Row],[المبلغ قبل الضريبة]]*VatRate,2)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" name="Column7">
+    <tableColumn id="7" name="الإجمالي">
       <calculatedColumnFormula>tblInv[[#This Row],[المبلغ قبل الضريبة]]+tblInv[[#This Row],[الضريبة]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" name="Column8">
+    <tableColumn id="8" name="مدة السداد">
       <calculatedColumnFormula>IFERROR(IF(INDEX(tblCustomers[مدة السداد],MATCH(tblInv[[#This Row],[كود العميل]],tblCustomers[كود العميل],0))="",DefaultTerms,INDEX(tblCustomers[مدة السداد],MATCH(tblInv[[#This Row],[كود العميل]],tblCustomers[كود العميل],0))),DefaultTerms)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" name="Column9">
+    <tableColumn id="9" name="تاريخ الاستحقاق">
       <calculatedColumnFormula>tblInv[[#This Row],[تاريخ الفاتورة]]+tblInv[[#This Row],[مدة السداد]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" name="Column10">
+    <tableColumn id="10" name="المحصّل">
       <calculatedColumnFormula>SUMIFS(tblRec[المبلغ],tblRec[رقم الفاتورة],tblInv[[#This Row],[رقم الفاتورة]],tblRec[التاريخ],"&lt;="&amp;AsOf)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" name="Column11">
+    <tableColumn id="11" name="المتبقي">
       <calculatedColumnFormula>IF(tblInv[[#This Row],[تاريخ الفاتورة]]&gt;AsOf,0,ROUND(tblInv[[#This Row],[الإجمالي]]-tblInv[[#This Row],[المحصّل]],2))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" name="Column12">
+    <tableColumn id="12" name="تاريخ الأساس">
       <calculatedColumnFormula>IF(AgingBasis="من تاريخ الفاتورة",tblInv[[#This Row],[تاريخ الفاتورة]],tblInv[[#This Row],[تاريخ الاستحقاق]])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" name="Column13">
+    <tableColumn id="13" name="أيام التأخير">
       <calculatedColumnFormula>IF(tblInv[[#This Row],[المتبقي]]&lt;=0,0,MAX(0,AsOf-tblInv[[#This Row],[تاريخ الأساس]]))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" name="Column14">
+    <tableColumn id="14" name="الفترة">
       <calculatedColumnFormula>IF(tblInv[[#This Row],[تاريخ الفاتورة]]&gt;AsOf,"بعد تاريخ التقرير",IF(tblInv[[#This Row],[المتبقي]]&lt;0,"⚠ تحصيل زائد",IF(tblInv[[#This Row],[المتبقي]]=0,"مسددة",IF(tblInv[[#This Row],[أيام التأخير]]=0,INDEX(tblBuckets[الفترة],1),LOOKUP(tblInv[[#This Row],[أيام التأخير]],tblBuckets[من يوم],tblBuckets[الفترة])))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" name="Column15">
+    <tableColumn id="15" name="الحالة">
       <calculatedColumnFormula>IF(tblInv[[#This Row],[تاريخ الفاتورة]]&gt;AsOf,"… بعد تاريخ التقرير",IF(tblInv[[#This Row],[المتبقي]]&lt;=0,"✓ مسددة",IF(tblInv[[#This Row],[المتبقي]]&lt;tblInv[[#This Row],[الإجمالي]],"◐ مسددة جزئياً",IF(tblInv[[#This Row],[أيام التأخير]]&gt;0,"● متأخرة","○ غير مستحقة"))))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" name="Column16"/>
+    <tableColumn id="16" name="ملاحظات"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showRowStripes="0"/>
 </table>
@@ -1300,17 +1268,17 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="tblRec" displayName="tblRec" ref="A4:I87" headerRowCount="1">
   <autoFilter ref="A4:I87"/>
   <tableColumns count="9">
-    <tableColumn id="1" name="Column1"/>
-    <tableColumn id="2" name="Column2"/>
-    <tableColumn id="3" name="Column3"/>
-    <tableColumn id="4" name="Column4">
+    <tableColumn id="1" name="رقم السند"/>
+    <tableColumn id="2" name="التاريخ"/>
+    <tableColumn id="3" name="كود العميل"/>
+    <tableColumn id="4" name="اسم العميل">
       <calculatedColumnFormula>IF(tblRec[[#This Row],[كود العميل]]="","",IFERROR(INDEX(tblCustomers[اسم العميل],MATCH(tblRec[[#This Row],[كود العميل]],tblCustomers[كود العميل],0)),"⚠ كود غير موجود"))</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" name="Column5"/>
-    <tableColumn id="6" name="Column6"/>
-    <tableColumn id="7" name="Column7"/>
-    <tableColumn id="8" name="Column8"/>
-    <tableColumn id="9" name="Column9">
+    <tableColumn id="5" name="رقم الفاتورة"/>
+    <tableColumn id="6" name="النوع"/>
+    <tableColumn id="7" name="المبلغ"/>
+    <tableColumn id="8" name="طريقة الدفع"/>
+    <tableColumn id="9" name="فحص">
       <calculatedColumnFormula>IF(tblRec[[#This Row],[رقم الفاتورة]]="","↺ دفعة غير مخصصة",IF(COUNTIF(tblInv[رقم الفاتورة],tblRec[[#This Row],[رقم الفاتورة]])=0,"⚠ رقم الفاتورة غير موجود",IF(COUNTIFS(tblInv[رقم الفاتورة],tblRec[[#This Row],[رقم الفاتورة]],tblInv[كود العميل],tblRec[[#This Row],[كود العميل]])=0,"⚠ الفاتورة مش لنفس العميل",IF(INDEX(tblInv[المتبقي],MATCH(tblRec[[#This Row],[رقم الفاتورة]],tblInv[رقم الفاتورة],0))&lt;0,"⚠ تحصيل أكبر من الفاتورة","✓"))))</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -4439,16 +4407,16 @@
   </conditionalFormatting>
   <dataValidations count="6">
     <dataValidation sqref="A5:A34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير صحيحة" error="الكود ده متكرر أو وصلت للحد الأقصى في النسخة المجانية (30 عميل)" type="custom" errorStyle="stop">
-      <formula1>=AND(COUNTIF($A$5:$A$534,A5)=1,ROW()&lt;=34)</formula1>
+      <formula1>AND(COUNTIF($A$5:$A$534,A5)=1,ROW()&lt;=34)</formula1>
     </dataValidation>
     <dataValidation sqref="C5:C34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير صحيحة" error="الرقم الضريبي لازم يكون 15 رقم" type="custom" errorStyle="stop">
-      <formula1>=AND(LEN(C5)=15,ISNUMBER(--C5))</formula1>
+      <formula1>AND(LEN(C5)=15,ISNUMBER(--C5))</formula1>
     </dataValidation>
     <dataValidation sqref="D5:D34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير مسموحة" error="من فضلك اختر قيمة من القائمة المنسدلة." type="list" errorStyle="warning">
-      <formula1>=CityList</formula1>
+      <formula1>CityList</formula1>
     </dataValidation>
     <dataValidation sqref="E5:E34" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير مسموحة" error="من فضلك اختر قيمة من القائمة المنسدلة." promptTitle="تنبيه" prompt="المندوب من القائمة (بتتعدل من الإعدادات)" type="list" errorStyle="stop">
-      <formula1>=RepList</formula1>
+      <formula1>RepList</formula1>
     </dataValidation>
     <dataValidation sqref="F5:F34" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير صحيحة" error="حد الائتمان رقم موجب" type="decimal" errorStyle="stop" operator="greaterThanOrEqual">
       <formula1>0</formula1>
@@ -12310,25 +12278,25 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="N5:N304">
     <cfRule type="expression" priority="8" dxfId="5">
-      <formula>N5=INDEX(tblBuckets[الفترة],1)</formula>
+      <formula>N5='الإعدادات'!$C$14</formula>
     </cfRule>
     <cfRule type="expression" priority="9" dxfId="6">
-      <formula>N5=INDEX(tblBuckets[الفترة],2)</formula>
+      <formula>N5='الإعدادات'!$C$15</formula>
     </cfRule>
     <cfRule type="expression" priority="10" dxfId="7">
-      <formula>N5=INDEX(tblBuckets[الفترة],3)</formula>
+      <formula>N5='الإعدادات'!$C$16</formula>
     </cfRule>
     <cfRule type="expression" priority="11" dxfId="8">
-      <formula>N5=INDEX(tblBuckets[الفترة],4)</formula>
+      <formula>N5='الإعدادات'!$C$17</formula>
     </cfRule>
     <cfRule type="expression" priority="12" dxfId="9">
-      <formula>N5=INDEX(tblBuckets[الفترة],5)</formula>
+      <formula>N5='الإعدادات'!$C$18</formula>
     </cfRule>
     <cfRule type="expression" priority="13" dxfId="10">
-      <formula>N5=INDEX(tblBuckets[الفترة],6)</formula>
+      <formula>N5='الإعدادات'!$C$19</formula>
     </cfRule>
     <cfRule type="expression" priority="14" dxfId="11">
-      <formula>N5=INDEX(tblBuckets[الفترة],7)</formula>
+      <formula>N5='الإعدادات'!$C$20</formula>
     </cfRule>
     <cfRule type="expression" priority="15" dxfId="0">
       <formula>LEFT(N5,1)="⚠"</formula>
@@ -12341,13 +12309,13 @@
   </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation sqref="A5:A304" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير صحيحة" error="رقم الفاتورة متكرر أو وصلت للحد الأقصى في النسخة المجانية (300 فاتورة)" type="custom" errorStyle="stop">
-      <formula1>=AND(COUNTIF($A$5:$A$1304,A5)=1,ROW()&lt;=304)</formula1>
+      <formula1>AND(COUNTIF($A$5:$A$1304,A5)=1,ROW()&lt;=304)</formula1>
     </dataValidation>
     <dataValidation sqref="B5:B304" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير صحيحة" error="لازم يكون تاريخ صحيح" type="date" errorStyle="stop" operator="greaterThan">
       <formula1>36526</formula1>
     </dataValidation>
     <dataValidation sqref="C5:C304" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير مسموحة" error="من فضلك اختر قيمة من القائمة المنسدلة." promptTitle="تنبيه" prompt="اختار كود العميل من القائمة" type="list" errorStyle="stop">
-      <formula1>=CustCodes</formula1>
+      <formula1>CustCodes</formula1>
     </dataValidation>
     <dataValidation sqref="E5:E304" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير صحيحة" error="المبلغ لازم يكون أكبر من صفر" type="decimal" errorStyle="stop" operator="greaterThan">
       <formula1>0</formula1>
@@ -15898,10 +15866,10 @@
       <formula1>36526</formula1>
     </dataValidation>
     <dataValidation sqref="C5:C604" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير مسموحة" error="من فضلك اختر قيمة من القائمة المنسدلة." promptTitle="تنبيه" prompt="اختار كود العميل" type="list" errorStyle="stop">
-      <formula1>=CustCodes</formula1>
+      <formula1>CustCodes</formula1>
     </dataValidation>
     <dataValidation sqref="E5:E604" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير مسموحة" error="من فضلك اختر قيمة من القائمة المنسدلة." promptTitle="تنبيه" prompt="رقم الفاتورة (فاضي = دفعة على الحساب)" type="list" errorStyle="warning">
-      <formula1>=InvNos</formula1>
+      <formula1>InvNos</formula1>
     </dataValidation>
     <dataValidation sqref="F5:F604" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير مسموحة" error="من فضلك اختر قيمة من القائمة المنسدلة." type="list" errorStyle="stop">
       <formula1>"تحصيل,إشعار دائن,خصم مسموح به,شطب دين"</formula1>
@@ -47422,10 +47390,10 @@
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="A5" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير مسموحة" error="من فضلك اختر قيمة من القائمة المنسدلة." promptTitle="تنبيه" prompt="فلتر بالمندوب" type="list" errorStyle="stop">
-      <formula1>=RepFilterList</formula1>
+      <formula1>RepFilterList</formula1>
     </dataValidation>
     <dataValidation sqref="C5" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="1" errorTitle="قيمة غير مسموحة" error="من فضلك اختر قيمة من القائمة المنسدلة." promptTitle="تنبيه" prompt="فلتر بالمدينة" type="list" errorStyle="stop">
-      <formula1>=CityFilterList</formula1>
+      <formula1>CityFilterList</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -47458,7 +47426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -47977,26 +47945,45 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="B19" s="110" t="inlineStr">
+    <row r="19">
+      <c r="H19" s="99" t="n">
+        <v>10</v>
+      </c>
+      <c r="I19" s="100">
+        <f>IFERROR(INDEX(tblCustomers[اسم العميل],MATCH(10,tblCustomers[ترتيب المتأخر],0)),"")</f>
+        <v/>
+      </c>
+      <c r="J19" s="100" t="n"/>
+      <c r="K19" s="100" t="n"/>
+      <c r="L19" s="101">
+        <f>IFERROR(INDEX(tblCustomers[المتأخر],MATCH(10,tblCustomers[ترتيب المتأخر],0)),0)</f>
+        <v/>
+      </c>
+      <c r="M19" s="102">
+        <f>IFERROR(INDEX(tblCustomers[أقدم فاتورة (يوم)],MATCH(10,tblCustomers[ترتيب المتأخر],0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="B22" s="110" t="inlineStr">
         <is>
           <t>🔒 متاح في النسخة الكاملة</t>
         </is>
       </c>
-      <c r="C19" s="111" t="n"/>
-      <c r="D19" s="111" t="n"/>
-      <c r="E19" s="111" t="n"/>
-      <c r="F19" s="111" t="n"/>
-      <c r="G19" s="111" t="n"/>
-      <c r="H19" s="111" t="n"/>
-      <c r="I19" s="111" t="n"/>
-      <c r="J19" s="111" t="n"/>
-      <c r="K19" s="111" t="n"/>
-      <c r="L19" s="111" t="n"/>
-      <c r="M19" s="110" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="112" t="inlineStr">
+      <c r="C22" s="110" t="n"/>
+      <c r="D22" s="110" t="n"/>
+      <c r="E22" s="110" t="n"/>
+      <c r="F22" s="110" t="n"/>
+      <c r="G22" s="110" t="n"/>
+      <c r="H22" s="110" t="n"/>
+      <c r="I22" s="110" t="n"/>
+      <c r="J22" s="110" t="n"/>
+      <c r="K22" s="110" t="n"/>
+      <c r="L22" s="110" t="n"/>
+      <c r="M22" s="110" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="111" t="inlineStr">
         <is>
           <t>• رسمة توزيع الأعمار بألوان الفترات   • رسمة أعلى 10 عملاء في المتأخر
 • قايمة متابعة التحصيل بالإجراء المقترح (واتساب / اتصال / خطاب / إيقاف توريد)
@@ -48004,87 +47991,87 @@
 • تقرير الأعمار بأي تاريخ سابق   • فترات ونسب قابلة للتعديل   • 500 عميل و5,000 فاتورة</t>
         </is>
       </c>
-      <c r="C20" s="112" t="n"/>
-      <c r="D20" s="112" t="n"/>
-      <c r="E20" s="112" t="n"/>
-      <c r="F20" s="112" t="n"/>
-      <c r="G20" s="112" t="n"/>
-      <c r="H20" s="112" t="n"/>
-      <c r="I20" s="112" t="n"/>
-      <c r="J20" s="112" t="n"/>
-      <c r="K20" s="112" t="n"/>
-      <c r="L20" s="112" t="n"/>
-      <c r="M20" s="112" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="112" t="n"/>
-      <c r="C21" s="112" t="n"/>
-      <c r="D21" s="112" t="n"/>
-      <c r="E21" s="112" t="n"/>
-      <c r="F21" s="112" t="n"/>
-      <c r="G21" s="112" t="n"/>
-      <c r="H21" s="112" t="n"/>
-      <c r="I21" s="112" t="n"/>
-      <c r="J21" s="112" t="n"/>
-      <c r="K21" s="112" t="n"/>
-      <c r="L21" s="112" t="n"/>
-      <c r="M21" s="112" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="112" t="n"/>
-      <c r="C22" s="112" t="n"/>
-      <c r="D22" s="112" t="n"/>
-      <c r="E22" s="112" t="n"/>
-      <c r="F22" s="112" t="n"/>
-      <c r="G22" s="112" t="n"/>
-      <c r="H22" s="112" t="n"/>
-      <c r="I22" s="112" t="n"/>
-      <c r="J22" s="112" t="n"/>
-      <c r="K22" s="112" t="n"/>
-      <c r="L22" s="112" t="n"/>
-      <c r="M22" s="112" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="112" t="n"/>
-      <c r="C23" s="112" t="n"/>
-      <c r="D23" s="112" t="n"/>
-      <c r="E23" s="112" t="n"/>
-      <c r="F23" s="112" t="n"/>
-      <c r="G23" s="112" t="n"/>
-      <c r="H23" s="112" t="n"/>
-      <c r="I23" s="112" t="n"/>
-      <c r="J23" s="112" t="n"/>
-      <c r="K23" s="112" t="n"/>
-      <c r="L23" s="112" t="n"/>
-      <c r="M23" s="112" t="n"/>
+      <c r="C23" s="111" t="n"/>
+      <c r="D23" s="111" t="n"/>
+      <c r="E23" s="111" t="n"/>
+      <c r="F23" s="111" t="n"/>
+      <c r="G23" s="111" t="n"/>
+      <c r="H23" s="111" t="n"/>
+      <c r="I23" s="111" t="n"/>
+      <c r="J23" s="111" t="n"/>
+      <c r="K23" s="111" t="n"/>
+      <c r="L23" s="111" t="n"/>
+      <c r="M23" s="111" t="n"/>
     </row>
     <row r="24">
-      <c r="B24" s="112" t="n"/>
-      <c r="C24" s="112" t="n"/>
-      <c r="D24" s="112" t="n"/>
-      <c r="E24" s="112" t="n"/>
-      <c r="F24" s="112" t="n"/>
-      <c r="G24" s="112" t="n"/>
-      <c r="H24" s="112" t="n"/>
-      <c r="I24" s="112" t="n"/>
-      <c r="J24" s="112" t="n"/>
-      <c r="K24" s="112" t="n"/>
-      <c r="L24" s="112" t="n"/>
-      <c r="M24" s="112" t="n"/>
+      <c r="B24" s="111" t="n"/>
+      <c r="C24" s="111" t="n"/>
+      <c r="D24" s="111" t="n"/>
+      <c r="E24" s="111" t="n"/>
+      <c r="F24" s="111" t="n"/>
+      <c r="G24" s="111" t="n"/>
+      <c r="H24" s="111" t="n"/>
+      <c r="I24" s="111" t="n"/>
+      <c r="J24" s="111" t="n"/>
+      <c r="K24" s="111" t="n"/>
+      <c r="L24" s="111" t="n"/>
+      <c r="M24" s="111" t="n"/>
     </row>
     <row r="25">
-      <c r="B25" s="112" t="n"/>
-      <c r="C25" s="112" t="n"/>
-      <c r="D25" s="112" t="n"/>
-      <c r="E25" s="112" t="n"/>
-      <c r="F25" s="112" t="n"/>
-      <c r="G25" s="112" t="n"/>
-      <c r="H25" s="112" t="n"/>
-      <c r="I25" s="112" t="n"/>
-      <c r="J25" s="112" t="n"/>
-      <c r="K25" s="112" t="n"/>
-      <c r="L25" s="112" t="n"/>
-      <c r="M25" s="112" t="n"/>
+      <c r="B25" s="111" t="n"/>
+      <c r="C25" s="111" t="n"/>
+      <c r="D25" s="111" t="n"/>
+      <c r="E25" s="111" t="n"/>
+      <c r="F25" s="111" t="n"/>
+      <c r="G25" s="111" t="n"/>
+      <c r="H25" s="111" t="n"/>
+      <c r="I25" s="111" t="n"/>
+      <c r="J25" s="111" t="n"/>
+      <c r="K25" s="111" t="n"/>
+      <c r="L25" s="111" t="n"/>
+      <c r="M25" s="111" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="111" t="n"/>
+      <c r="C26" s="111" t="n"/>
+      <c r="D26" s="111" t="n"/>
+      <c r="E26" s="111" t="n"/>
+      <c r="F26" s="111" t="n"/>
+      <c r="G26" s="111" t="n"/>
+      <c r="H26" s="111" t="n"/>
+      <c r="I26" s="111" t="n"/>
+      <c r="J26" s="111" t="n"/>
+      <c r="K26" s="111" t="n"/>
+      <c r="L26" s="111" t="n"/>
+      <c r="M26" s="111" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="111" t="n"/>
+      <c r="C27" s="111" t="n"/>
+      <c r="D27" s="111" t="n"/>
+      <c r="E27" s="111" t="n"/>
+      <c r="F27" s="111" t="n"/>
+      <c r="G27" s="111" t="n"/>
+      <c r="H27" s="111" t="n"/>
+      <c r="I27" s="111" t="n"/>
+      <c r="J27" s="111" t="n"/>
+      <c r="K27" s="111" t="n"/>
+      <c r="L27" s="111" t="n"/>
+      <c r="M27" s="111" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="111" t="n"/>
+      <c r="C28" s="111" t="n"/>
+      <c r="D28" s="111" t="n"/>
+      <c r="E28" s="111" t="n"/>
+      <c r="F28" s="111" t="n"/>
+      <c r="G28" s="111" t="n"/>
+      <c r="H28" s="111" t="n"/>
+      <c r="I28" s="111" t="n"/>
+      <c r="J28" s="111" t="n"/>
+      <c r="K28" s="111" t="n"/>
+      <c r="L28" s="111" t="n"/>
+      <c r="M28" s="111" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
@@ -48109,9 +48096,7 @@
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="E10:F10"/>
     <mergeCell ref="I14:K14"/>
-    <mergeCell ref="B19:M19"/>
     <mergeCell ref="F5:G5"/>
-    <mergeCell ref="B20:M25"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="E13:F13"/>
     <mergeCell ref="L5:M5"/>
@@ -48133,7 +48118,9 @@
     <mergeCell ref="E16:F16"/>
     <mergeCell ref="L6:M6"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B23:M28"/>
     <mergeCell ref="D5:E5"/>
+    <mergeCell ref="B22:M22"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="B12:D12"/>
   </mergeCells>

</xml_diff>